<commit_message>
Implementasi Single Point Crossover & Penerapan Soft Constraint SC3 (Pembatasan Piket Berturut-turut)
</commit_message>
<xml_diff>
--- a/results/schedules/jadwal_gsk08.xlsx
+++ b/results/schedules/jadwal_gsk08.xlsx
@@ -31,11 +31,11 @@
       <sz val="11"/>
     </font>
     <font>
+      <color rgb="00A7F3D0"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFD666"/>
-    </font>
-    <font>
-      <color rgb="00A7F3D0"/>
     </font>
     <font>
       <i val="1"/>
@@ -57,14 +57,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004A1215"/>
-        <bgColor rgb="004A1215"/>
+        <fgColor rgb="00064E3B"/>
+        <bgColor rgb="00064E3B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00064E3B"/>
-        <bgColor rgb="00064E3B"/>
+        <fgColor rgb="004A1215"/>
+        <bgColor rgb="004A1215"/>
       </patternFill>
     </fill>
     <fill>
@@ -567,35 +567,35 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -617,39 +617,39 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -669,39 +669,39 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -723,35 +723,35 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -775,37 +775,37 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -827,35 +827,35 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -877,37 +877,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -929,37 +929,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>
@@ -983,35 +983,35 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1035,35 +1035,35 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1085,39 +1085,39 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -1139,37 +1139,37 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -1191,35 +1191,35 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1241,39 +1241,39 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -1295,35 +1295,35 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1347,35 +1347,35 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1397,39 +1397,39 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -1451,35 +1451,35 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1501,37 +1501,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1553,37 +1553,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1605,39 +1605,39 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -1659,35 +1659,35 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1709,37 +1709,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1761,37 +1761,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1813,39 +1813,39 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -1865,37 +1865,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -1917,39 +1917,39 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -1971,35 +1971,35 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2021,37 +2021,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2073,37 +2073,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>
@@ -2125,37 +2125,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2177,37 +2177,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2231,35 +2231,35 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2281,37 +2281,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2333,39 +2333,39 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -2385,37 +2385,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2437,37 +2437,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2489,37 +2489,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2541,37 +2541,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2593,37 +2593,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2645,37 +2645,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2697,37 +2697,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2749,37 +2749,37 @@
           <t>JUMAT</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2803,35 +2803,35 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I45" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2853,37 +2853,37 @@
           <t>RABU</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -2905,37 +2905,37 @@
           <t>MINGGU</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J47" s="3" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>
@@ -2957,37 +2957,37 @@
           <t>MINGGU</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J48" s="3" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>
@@ -3009,37 +3009,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J49" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -3061,37 +3061,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J50" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -3113,37 +3113,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -3165,37 +3165,37 @@
           <t>MINGGU</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J52" s="3" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>
@@ -3219,35 +3219,35 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I53" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J53" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -3269,37 +3269,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J54" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -3323,37 +3323,37 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -3373,37 +3373,37 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr">
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
         <is>
           <t>PIKET</t>
         </is>
@@ -3425,37 +3425,37 @@
           <t>MINGGU</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J57" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
         <is>
           <t>LIBUR</t>
         </is>

</xml_diff>